<commit_message>
feat: Added new test types
</commit_message>
<xml_diff>
--- a/resources/commonlab.xlsx
+++ b/resources/commonlab.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="442">
   <si>
     <t>uuid</t>
   </si>
@@ -1288,6 +1288,93 @@
   </si>
   <si>
     <t>95b09185-3928-11ee-9784-e86a64440f18</t>
+  </si>
+  <si>
+    <t>XPERT ULTRA</t>
+  </si>
+  <si>
+    <t>c91fb03b-acaf-4a3c-9a5b-3d32e4ac4d34</t>
+  </si>
+  <si>
+    <t>159f8b31-0c0a-4377-bea9-667a72a949b7</t>
+  </si>
+  <si>
+    <t>cedb082c-3a94-48f6-a192-fda9f2c48afd</t>
+  </si>
+  <si>
+    <t>XPERT ULTRA MTB BURDEN</t>
+  </si>
+  <si>
+    <t>ab70a74d-2bcd-4deb-abe7-d3dc9058edaf</t>
+  </si>
+  <si>
+    <t>3fb27302-f1ca-477a-9306-58bba806cfd8</t>
+  </si>
+  <si>
+    <t>686387e4-af27-4442-af41-395e72f1f712</t>
+  </si>
+  <si>
+    <t>ec9b4609-7ea5-461e-9aa6-bd515d230d52</t>
+  </si>
+  <si>
+    <t>479844a7-745f-4d40-9fff-dd254dfd8935</t>
+  </si>
+  <si>
+    <t>b28d58fc-a765-4a63-9d43-538c1880a413</t>
+  </si>
+  <si>
+    <t>e69a0ce4-18c9-49f9-bcfb-713447214933</t>
+  </si>
+  <si>
+    <t>fd5ef525-8f47-4553-836b-a00289e2e2a0</t>
+  </si>
+  <si>
+    <t>XPERT XDR</t>
+  </si>
+  <si>
+    <t>f516fc8a-2a06-4ffa-bbcb-1f69d855dd14</t>
+  </si>
+  <si>
+    <t>304cf8f8-2424-4070-a7aa-721b971d0894</t>
+  </si>
+  <si>
+    <t>a3d9d7f6-0cea-4fe9-968e-5778438e8226</t>
+  </si>
+  <si>
+    <t>89d6f422-6653-413f-9d44-be07095d383e</t>
+  </si>
+  <si>
+    <t>f6ca29a8-c6d5-49b9-b25d-e0a1e20de760</t>
+  </si>
+  <si>
+    <t>KM/AM/CM RESULT</t>
+  </si>
+  <si>
+    <t>6e350688-a9e8-4685-b614-b5951542c6d6</t>
+  </si>
+  <si>
+    <t>ETHIONAMIDE RESULT</t>
+  </si>
+  <si>
+    <t>f4cde26f-614b-4015-8c20-497bc90f7de1</t>
+  </si>
+  <si>
+    <t>1ad71659-6d1d-4e86-a489-8c12e70b13a9</t>
+  </si>
+  <si>
+    <t>c48f9814-6c04-471b-adda-713625e6678e</t>
+  </si>
+  <si>
+    <t>97866288-9749-476d-862f-dd9a09076186</t>
+  </si>
+  <si>
+    <t>de67a5c3-a093-419e-96ea-f376530824f5</t>
+  </si>
+  <si>
+    <t>75a82d0c-a2dc-49e0-9d27-3a42950713df</t>
+  </si>
+  <si>
+    <t>f399e490-ed5a-474f-a755-63d22092e05f</t>
   </si>
 </sst>
 </file>
@@ -1979,7 +2066,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91536433-8730-4EA0-BCCE-0E80DA08A6A5}">
-  <dimension ref="A1:Q205"/>
+  <dimension ref="A1:Q227"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
@@ -11564,9 +11651,1087 @@
         <v>360</v>
       </c>
     </row>
+    <row r="206" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206">
+        <v>5</v>
+      </c>
+      <c r="C206" t="s">
+        <v>34</v>
+      </c>
+      <c r="D206" t="s">
+        <v>35</v>
+      </c>
+      <c r="E206">
+        <v>0</v>
+      </c>
+      <c r="F206">
+        <v>1</v>
+      </c>
+      <c r="G206" t="s">
+        <v>36</v>
+      </c>
+      <c r="H206">
+        <v>109</v>
+      </c>
+      <c r="I206" t="str">
+        <f>C206 &amp; " " &amp;L206</f>
+        <v xml:space="preserve">APPEARANCE OF SPECIMEN XPERT ULTRA</v>
+      </c>
+      <c r="J206" t="s">
+        <v>37</v>
+      </c>
+      <c r="K206"/>
+      <c r="L206" t="s">
+        <v>413</v>
+      </c>
+      <c r="M206"/>
+      <c r="N206">
+        <v>1</v>
+      </c>
+      <c r="O206" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P206">
+        <v>0</v>
+      </c>
+      <c r="Q206" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="207" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>206</v>
+      </c>
+      <c r="B207">
+        <v>5</v>
+      </c>
+      <c r="C207" t="s">
+        <v>51</v>
+      </c>
+      <c r="D207" t="s">
+        <v>35</v>
+      </c>
+      <c r="E207">
+        <v>0</v>
+      </c>
+      <c r="F207">
+        <v>1</v>
+      </c>
+      <c r="G207" t="s">
+        <v>52</v>
+      </c>
+      <c r="H207">
+        <v>110</v>
+      </c>
+      <c r="I207" t="str">
+        <f>C207 &amp; " " &amp;L207</f>
+        <v xml:space="preserve">MTB RESULT XPERT ULTRA</v>
+      </c>
+      <c r="J207" t="s">
+        <v>37</v>
+      </c>
+      <c r="K207"/>
+      <c r="L207" t="s">
+        <v>413</v>
+      </c>
+      <c r="M207"/>
+      <c r="N207">
+        <v>1</v>
+      </c>
+      <c r="O207" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P207">
+        <v>0</v>
+      </c>
+      <c r="Q207" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="208" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>207</v>
+      </c>
+      <c r="B208">
+        <v>5</v>
+      </c>
+      <c r="C208" t="s">
+        <v>85</v>
+      </c>
+      <c r="D208" t="s">
+        <v>44</v>
+      </c>
+      <c r="E208">
+        <v>0</v>
+      </c>
+      <c r="F208">
+        <v>1</v>
+      </c>
+      <c r="G208" t="s">
+        <v>45</v>
+      </c>
+      <c r="H208">
+        <v>111</v>
+      </c>
+      <c r="I208" t="str">
+        <f>C208 &amp; " " &amp;L208</f>
+        <v xml:space="preserve">ERROR CODE XPERT ULTRA</v>
+      </c>
+      <c r="J208" t="s">
+        <v>46</v>
+      </c>
+      <c r="K208"/>
+      <c r="L208" t="s">
+        <v>413</v>
+      </c>
+      <c r="M208"/>
+      <c r="N208">
+        <v>1</v>
+      </c>
+      <c r="O208" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P208">
+        <v>0</v>
+      </c>
+      <c r="Q208" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="209" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>208</v>
+      </c>
+      <c r="B209">
+        <v>5</v>
+      </c>
+      <c r="C209" t="s">
+        <v>417</v>
+      </c>
+      <c r="D209" t="s">
+        <v>35</v>
+      </c>
+      <c r="E209">
+        <v>0</v>
+      </c>
+      <c r="F209">
+        <v>1</v>
+      </c>
+      <c r="G209" t="s">
+        <v>418</v>
+      </c>
+      <c r="H209">
+        <v>112</v>
+      </c>
+      <c r="I209" t="str">
+        <f>C209 &amp; " " &amp;L209</f>
+        <v xml:space="preserve">XPERT ULTRA MTB BURDEN XPERT ULTRA</v>
+      </c>
+      <c r="J209" t="s">
+        <v>37</v>
+      </c>
+      <c r="K209"/>
+      <c r="L209" t="s">
+        <v>413</v>
+      </c>
+      <c r="M209"/>
+      <c r="N209">
+        <v>1</v>
+      </c>
+      <c r="O209" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P209">
+        <v>0</v>
+      </c>
+      <c r="Q209" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" s="1">
+        <v>5</v>
+      </c>
+      <c r="C210" t="s">
+        <v>171</v>
+      </c>
+      <c r="D210" t="s">
+        <v>35</v>
+      </c>
+      <c r="E210">
+        <v>0</v>
+      </c>
+      <c r="F210">
+        <v>1</v>
+      </c>
+      <c r="G210" t="s">
+        <v>62</v>
+      </c>
+      <c r="H210">
+        <v>113</v>
+      </c>
+      <c r="I210" t="str">
+        <f>C210 &amp; " " &amp;L210</f>
+        <v xml:space="preserve">RIFAMPICIN RESULT XPERT ULTRA</v>
+      </c>
+      <c r="J210" t="s">
+        <v>37</v>
+      </c>
+      <c r="L210" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="N210">
+        <v>1</v>
+      </c>
+      <c r="O210" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P210">
+        <v>0</v>
+      </c>
+      <c r="Q210" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="211" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211">
+        <v>5</v>
+      </c>
+      <c r="C211" t="s">
+        <v>81</v>
+      </c>
+      <c r="D211" t="s">
+        <v>39</v>
+      </c>
+      <c r="E211">
+        <v>0</v>
+      </c>
+      <c r="F211">
+        <v>1</v>
+      </c>
+      <c r="G211"/>
+      <c r="H211">
+        <v>114</v>
+      </c>
+      <c r="I211" t="str">
+        <f>C211 &amp; " " &amp;L211</f>
+        <v xml:space="preserve">TUBERCULOSIS TEST RESULT DATE XPERT ULTRA</v>
+      </c>
+      <c r="J211" t="s">
+        <v>41</v>
+      </c>
+      <c r="K211"/>
+      <c r="L211" t="s">
+        <v>413</v>
+      </c>
+      <c r="M211"/>
+      <c r="N211">
+        <v>1</v>
+      </c>
+      <c r="O211" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P211">
+        <v>0</v>
+      </c>
+      <c r="Q211" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="212" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212">
+        <v>5</v>
+      </c>
+      <c r="C212" t="s">
+        <v>279</v>
+      </c>
+      <c r="D212" t="s">
+        <v>39</v>
+      </c>
+      <c r="E212">
+        <v>0</v>
+      </c>
+      <c r="F212">
+        <v>1</v>
+      </c>
+      <c r="G212"/>
+      <c r="H212">
+        <v>115</v>
+      </c>
+      <c r="I212" t="str">
+        <f>C212 &amp; " " &amp;L212</f>
+        <v xml:space="preserve">DATE OF SENDING TO CULTURE XPERT ULTRA</v>
+      </c>
+      <c r="J212" t="s">
+        <v>41</v>
+      </c>
+      <c r="K212"/>
+      <c r="L212" t="s">
+        <v>413</v>
+      </c>
+      <c r="M212"/>
+      <c r="N212">
+        <v>1</v>
+      </c>
+      <c r="O212" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P212">
+        <v>0</v>
+      </c>
+      <c r="Q212" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="213" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213">
+        <v>5</v>
+      </c>
+      <c r="C213" t="s">
+        <v>280</v>
+      </c>
+      <c r="D213" t="s">
+        <v>39</v>
+      </c>
+      <c r="E213">
+        <v>0</v>
+      </c>
+      <c r="F213">
+        <v>1</v>
+      </c>
+      <c r="G213"/>
+      <c r="H213">
+        <v>116</v>
+      </c>
+      <c r="I213" t="str">
+        <f>C213 &amp; " " &amp;L213</f>
+        <v xml:space="preserve">DATE OF SENDING TO DST XPERT ULTRA</v>
+      </c>
+      <c r="J213" t="s">
+        <v>41</v>
+      </c>
+      <c r="K213"/>
+      <c r="L213" t="s">
+        <v>413</v>
+      </c>
+      <c r="M213"/>
+      <c r="N213">
+        <v>1</v>
+      </c>
+      <c r="O213" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P213">
+        <v>0</v>
+      </c>
+      <c r="Q213" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="214" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214">
+        <v>5</v>
+      </c>
+      <c r="C214" t="s">
+        <v>282</v>
+      </c>
+      <c r="D214" t="s">
+        <v>35</v>
+      </c>
+      <c r="E214">
+        <v>0</v>
+      </c>
+      <c r="F214">
+        <v>1</v>
+      </c>
+      <c r="G214" t="s">
+        <v>295</v>
+      </c>
+      <c r="H214">
+        <v>117</v>
+      </c>
+      <c r="I214" t="str">
+        <f>C214 &amp; " " &amp;L214</f>
+        <v xml:space="preserve">SENT TO CULTURE XPERT ULTRA</v>
+      </c>
+      <c r="J214" t="s">
+        <v>37</v>
+      </c>
+      <c r="K214"/>
+      <c r="L214" t="s">
+        <v>413</v>
+      </c>
+      <c r="M214"/>
+      <c r="N214">
+        <v>1</v>
+      </c>
+      <c r="O214" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P214">
+        <v>0</v>
+      </c>
+      <c r="Q214" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="215" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215">
+        <v>5</v>
+      </c>
+      <c r="C215" t="s">
+        <v>281</v>
+      </c>
+      <c r="D215" t="s">
+        <v>35</v>
+      </c>
+      <c r="E215">
+        <v>0</v>
+      </c>
+      <c r="F215">
+        <v>1</v>
+      </c>
+      <c r="G215" t="s">
+        <v>294</v>
+      </c>
+      <c r="H215">
+        <v>118</v>
+      </c>
+      <c r="I215" t="str">
+        <f>C215 &amp; " " &amp;L215</f>
+        <v xml:space="preserve">SENT TO DST XPERT ULTRA</v>
+      </c>
+      <c r="J215" t="s">
+        <v>37</v>
+      </c>
+      <c r="K215"/>
+      <c r="L215" t="s">
+        <v>413</v>
+      </c>
+      <c r="M215"/>
+      <c r="N215">
+        <v>1</v>
+      </c>
+      <c r="O215" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P215">
+        <v>0</v>
+      </c>
+      <c r="Q215" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="216" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216">
+        <v>5</v>
+      </c>
+      <c r="C216" t="s">
+        <v>34</v>
+      </c>
+      <c r="D216" t="s">
+        <v>35</v>
+      </c>
+      <c r="E216">
+        <v>0</v>
+      </c>
+      <c r="F216">
+        <v>1</v>
+      </c>
+      <c r="G216" t="s">
+        <v>36</v>
+      </c>
+      <c r="H216">
+        <v>119</v>
+      </c>
+      <c r="I216" t="str">
+        <f>C216 &amp; " " &amp;L216</f>
+        <v xml:space="preserve">APPEARANCE OF SPECIMEN XPERT XDR</v>
+      </c>
+      <c r="J216" t="s">
+        <v>37</v>
+      </c>
+      <c r="K216"/>
+      <c r="L216" t="s">
+        <v>426</v>
+      </c>
+      <c r="M216"/>
+      <c r="N216">
+        <v>1</v>
+      </c>
+      <c r="O216" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P216">
+        <v>0</v>
+      </c>
+      <c r="Q216" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="217" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217">
+        <v>5</v>
+      </c>
+      <c r="C217" t="s">
+        <v>51</v>
+      </c>
+      <c r="D217" t="s">
+        <v>35</v>
+      </c>
+      <c r="E217">
+        <v>0</v>
+      </c>
+      <c r="F217">
+        <v>1</v>
+      </c>
+      <c r="G217" t="s">
+        <v>52</v>
+      </c>
+      <c r="H217">
+        <v>120</v>
+      </c>
+      <c r="I217" t="str">
+        <f>C217 &amp; " " &amp;L217</f>
+        <v xml:space="preserve">MTB RESULT XPERT XDR</v>
+      </c>
+      <c r="J217" t="s">
+        <v>37</v>
+      </c>
+      <c r="K217"/>
+      <c r="L217" t="s">
+        <v>426</v>
+      </c>
+      <c r="M217"/>
+      <c r="N217">
+        <v>1</v>
+      </c>
+      <c r="O217" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P217">
+        <v>0</v>
+      </c>
+      <c r="Q217" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="218" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218">
+        <v>5</v>
+      </c>
+      <c r="C218" t="s">
+        <v>85</v>
+      </c>
+      <c r="D218" t="s">
+        <v>44</v>
+      </c>
+      <c r="E218">
+        <v>0</v>
+      </c>
+      <c r="F218">
+        <v>1</v>
+      </c>
+      <c r="G218" t="s">
+        <v>45</v>
+      </c>
+      <c r="H218">
+        <v>121</v>
+      </c>
+      <c r="I218" t="str">
+        <f>C218 &amp; " " &amp;L218</f>
+        <v xml:space="preserve">ERROR CODE XPERT XDR</v>
+      </c>
+      <c r="J218" t="s">
+        <v>46</v>
+      </c>
+      <c r="K218"/>
+      <c r="L218" t="s">
+        <v>426</v>
+      </c>
+      <c r="M218"/>
+      <c r="N218">
+        <v>1</v>
+      </c>
+      <c r="O218" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P218">
+        <v>0</v>
+      </c>
+      <c r="Q218" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>218</v>
+      </c>
+      <c r="B219" s="1">
+        <v>5</v>
+      </c>
+      <c r="C219" t="s">
+        <v>170</v>
+      </c>
+      <c r="D219" t="s">
+        <v>35</v>
+      </c>
+      <c r="E219">
+        <v>0</v>
+      </c>
+      <c r="F219">
+        <v>1</v>
+      </c>
+      <c r="G219" t="s">
+        <v>88</v>
+      </c>
+      <c r="H219">
+        <v>122</v>
+      </c>
+      <c r="I219" t="str">
+        <f>C219 &amp; " " &amp;L219</f>
+        <v xml:space="preserve">ISONIAZID RESULT XPERT XDR</v>
+      </c>
+      <c r="J219" t="s">
+        <v>37</v>
+      </c>
+      <c r="L219" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="N219">
+        <v>1</v>
+      </c>
+      <c r="O219" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P219">
+        <v>0</v>
+      </c>
+      <c r="Q219" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220">
+        <v>5</v>
+      </c>
+      <c r="C220" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="D220" t="s">
+        <v>35</v>
+      </c>
+      <c r="E220">
+        <v>0</v>
+      </c>
+      <c r="F220">
+        <v>1</v>
+      </c>
+      <c r="G220" t="s">
+        <v>289</v>
+      </c>
+      <c r="H220">
+        <v>123</v>
+      </c>
+      <c r="I220" t="str">
+        <f>C220 &amp; " " &amp;L220</f>
+        <v xml:space="preserve">MOX/OFX RESULT XPERT XDR</v>
+      </c>
+      <c r="J220" t="s">
+        <v>37</v>
+      </c>
+      <c r="L220" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="N220">
+        <v>1</v>
+      </c>
+      <c r="O220" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P220">
+        <v>0</v>
+      </c>
+      <c r="Q220" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="221" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>220</v>
+      </c>
+      <c r="B221">
+        <v>5</v>
+      </c>
+      <c r="C221" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D221" t="s">
+        <v>35</v>
+      </c>
+      <c r="E221">
+        <v>0</v>
+      </c>
+      <c r="F221">
+        <v>1</v>
+      </c>
+      <c r="G221" t="s">
+        <v>288</v>
+      </c>
+      <c r="H221">
+        <v>124</v>
+      </c>
+      <c r="I221" t="str">
+        <f>C221 &amp; " " &amp;L221</f>
+        <v xml:space="preserve">KM/AM/CM RESULT XPERT XDR</v>
+      </c>
+      <c r="J221" t="s">
+        <v>37</v>
+      </c>
+      <c r="L221" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="N221">
+        <v>1</v>
+      </c>
+      <c r="O221" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P221">
+        <v>0</v>
+      </c>
+      <c r="Q221" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="222" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>221</v>
+      </c>
+      <c r="B222" s="1">
+        <v>5</v>
+      </c>
+      <c r="C222" t="s">
+        <v>434</v>
+      </c>
+      <c r="D222" t="s">
+        <v>35</v>
+      </c>
+      <c r="E222">
+        <v>0</v>
+      </c>
+      <c r="F222">
+        <v>1</v>
+      </c>
+      <c r="G222" t="s">
+        <v>435</v>
+      </c>
+      <c r="H222">
+        <v>125</v>
+      </c>
+      <c r="I222" t="str">
+        <f>C222 &amp; " " &amp;L222</f>
+        <v xml:space="preserve">ETHIONAMIDE RESULT XPERT XDR</v>
+      </c>
+      <c r="J222" t="s">
+        <v>37</v>
+      </c>
+      <c r="L222" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="N222">
+        <v>1</v>
+      </c>
+      <c r="O222" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P222">
+        <v>0</v>
+      </c>
+      <c r="Q222" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="223" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>222</v>
+      </c>
+      <c r="B223">
+        <v>5</v>
+      </c>
+      <c r="C223" t="s">
+        <v>81</v>
+      </c>
+      <c r="D223" t="s">
+        <v>39</v>
+      </c>
+      <c r="E223">
+        <v>0</v>
+      </c>
+      <c r="F223">
+        <v>1</v>
+      </c>
+      <c r="G223"/>
+      <c r="H223">
+        <v>126</v>
+      </c>
+      <c r="I223" t="str">
+        <f>C223 &amp; " " &amp;L223</f>
+        <v xml:space="preserve">TUBERCULOSIS TEST RESULT DATE XPERT XDR</v>
+      </c>
+      <c r="J223" t="s">
+        <v>41</v>
+      </c>
+      <c r="K223"/>
+      <c r="L223" t="s">
+        <v>426</v>
+      </c>
+      <c r="M223"/>
+      <c r="N223">
+        <v>1</v>
+      </c>
+      <c r="O223" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P223">
+        <v>0</v>
+      </c>
+      <c r="Q223" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="224" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>223</v>
+      </c>
+      <c r="B224">
+        <v>5</v>
+      </c>
+      <c r="C224" t="s">
+        <v>279</v>
+      </c>
+      <c r="D224" t="s">
+        <v>39</v>
+      </c>
+      <c r="E224">
+        <v>0</v>
+      </c>
+      <c r="F224">
+        <v>1</v>
+      </c>
+      <c r="G224"/>
+      <c r="H224">
+        <v>127</v>
+      </c>
+      <c r="I224" t="str">
+        <f>C224 &amp; " " &amp;L224</f>
+        <v xml:space="preserve">DATE OF SENDING TO CULTURE XPERT XDR</v>
+      </c>
+      <c r="J224" t="s">
+        <v>41</v>
+      </c>
+      <c r="K224"/>
+      <c r="L224" t="s">
+        <v>426</v>
+      </c>
+      <c r="M224"/>
+      <c r="N224">
+        <v>1</v>
+      </c>
+      <c r="O224" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P224">
+        <v>0</v>
+      </c>
+      <c r="Q224" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="225" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>224</v>
+      </c>
+      <c r="B225">
+        <v>5</v>
+      </c>
+      <c r="C225" t="s">
+        <v>280</v>
+      </c>
+      <c r="D225" t="s">
+        <v>39</v>
+      </c>
+      <c r="E225">
+        <v>0</v>
+      </c>
+      <c r="F225">
+        <v>1</v>
+      </c>
+      <c r="G225"/>
+      <c r="H225">
+        <v>128</v>
+      </c>
+      <c r="I225" t="str">
+        <f>C225 &amp; " " &amp;L225</f>
+        <v xml:space="preserve">DATE OF SENDING TO DST XPERT XDR</v>
+      </c>
+      <c r="J225" t="s">
+        <v>41</v>
+      </c>
+      <c r="K225"/>
+      <c r="L225" t="s">
+        <v>426</v>
+      </c>
+      <c r="M225"/>
+      <c r="N225">
+        <v>1</v>
+      </c>
+      <c r="O225" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P225">
+        <v>0</v>
+      </c>
+      <c r="Q225" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="226" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226">
+        <v>5</v>
+      </c>
+      <c r="C226" t="s">
+        <v>282</v>
+      </c>
+      <c r="D226" t="s">
+        <v>35</v>
+      </c>
+      <c r="E226">
+        <v>0</v>
+      </c>
+      <c r="F226">
+        <v>1</v>
+      </c>
+      <c r="G226" t="s">
+        <v>295</v>
+      </c>
+      <c r="H226">
+        <v>129</v>
+      </c>
+      <c r="I226" t="str">
+        <f>C226 &amp; " " &amp;L226</f>
+        <v xml:space="preserve">SENT TO CULTURE XPERT XDR</v>
+      </c>
+      <c r="J226" t="s">
+        <v>37</v>
+      </c>
+      <c r="K226"/>
+      <c r="L226" t="s">
+        <v>426</v>
+      </c>
+      <c r="M226"/>
+      <c r="N226">
+        <v>1</v>
+      </c>
+      <c r="O226" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P226">
+        <v>0</v>
+      </c>
+      <c r="Q226" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="227" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227">
+        <v>5</v>
+      </c>
+      <c r="C227" t="s">
+        <v>281</v>
+      </c>
+      <c r="D227" t="s">
+        <v>35</v>
+      </c>
+      <c r="E227">
+        <v>0</v>
+      </c>
+      <c r="F227">
+        <v>1</v>
+      </c>
+      <c r="G227" t="s">
+        <v>294</v>
+      </c>
+      <c r="H227">
+        <v>130</v>
+      </c>
+      <c r="I227" t="str">
+        <f>C227 &amp; " " &amp;L227</f>
+        <v xml:space="preserve">SENT TO DST XPERT XDR</v>
+      </c>
+      <c r="J227" t="s">
+        <v>37</v>
+      </c>
+      <c r="K227"/>
+      <c r="L227" t="s">
+        <v>426</v>
+      </c>
+      <c r="M227"/>
+      <c r="N227">
+        <v>1</v>
+      </c>
+      <c r="O227" s="4">
+        <v>46313</v>
+      </c>
+      <c r="P227">
+        <v>0</v>
+      </c>
+      <c r="Q227" t="s">
+        <v>441</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q205" xr:uid="{91536433-8730-4EA0-BCCE-0E80DA08A6A5}"/>
-  <conditionalFormatting sqref="Q2:Q205">
+  <autoFilter ref="A1:Q227" xr:uid="{91536433-8730-4EA0-BCCE-0E80DA08A6A5}"/>
+  <conditionalFormatting sqref="Q2:Q227">
     <cfRule type="duplicateValues" dxfId="0" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refresh lab and concept mappings
Updated the common lab reference workbook and the concept mapping spreadsheet used by the ETL pipeline.
</commit_message>
<xml_diff>
--- a/resources/commonlab.xlsx
+++ b/resources/commonlab.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="474">
   <si>
     <t>uuid</t>
   </si>
@@ -1375,6 +1375,102 @@
   </si>
   <si>
     <t>f399e490-ed5a-474f-a755-63d22092e05f</t>
+  </si>
+  <si>
+    <t>3bb32248-55b5-4513-a681-2f753646a543</t>
+  </si>
+  <si>
+    <t>XPERT ULTRA RESULT</t>
+  </si>
+  <si>
+    <t>0075b266-74f3-4ed7-a822-369ffe92c7b2</t>
+  </si>
+  <si>
+    <t>TEST NUMBER</t>
+  </si>
+  <si>
+    <t>Regex=[0-9A-Za-z/-]*</t>
+  </si>
+  <si>
+    <t>0d35f6db-f13a-4c4a-9a9a-0fc14d2167d2</t>
+  </si>
+  <si>
+    <t>LAB</t>
+  </si>
+  <si>
+    <t>17b6e353-8488-4fb2-b100-6574b41d15be</t>
+  </si>
+  <si>
+    <t>736346b3-54c5-491e-95db-0c76b65630c3</t>
+  </si>
+  <si>
+    <t>fc66e7d3-632b-4fda-9eb6-b64844228412</t>
+  </si>
+  <si>
+    <t>XPERT XDR RESULT</t>
+  </si>
+  <si>
+    <t>9e2b0d1b-9bb3-4761-bf84-0668bed74e92</t>
+  </si>
+  <si>
+    <t>ISONIAZID (H)</t>
+  </si>
+  <si>
+    <t>e03067c3-2e0d-4b27-aaa7-0a21683e2543</t>
+  </si>
+  <si>
+    <t>9ed60f80-acf9-4ef8-930e-f02be2a7aeb5</t>
+  </si>
+  <si>
+    <t>FLUOROQUINOLONES (FQ)</t>
+  </si>
+  <si>
+    <t>32342299-8bc1-4eb2-a02e-797140ee763e</t>
+  </si>
+  <si>
+    <t>42630a36-b380-4fcd-9ef3-12e2efb8fad3</t>
+  </si>
+  <si>
+    <t>AMIKACIN (AM)</t>
+  </si>
+  <si>
+    <t>ab9ebf0d-767b-4319-abdb-86bede788c20</t>
+  </si>
+  <si>
+    <t>c202c6e1-0057-4ff2-84cb-8d53d86e5fc2</t>
+  </si>
+  <si>
+    <t>CAPREOMYCIN (CM)</t>
+  </si>
+  <si>
+    <t>84156f85-6d51-43ae-8dfd-90563027b9b8</t>
+  </si>
+  <si>
+    <t>34b96045-b2c1-4165-9390-3dd12153e1f5</t>
+  </si>
+  <si>
+    <t>KANAMYCIN (KM)</t>
+  </si>
+  <si>
+    <t>bdf9767b-745e-4d67-9c91-786030507a16</t>
+  </si>
+  <si>
+    <t>8a2f3e93-aa83-44f9-abc3-a4a5eeadb8c9</t>
+  </si>
+  <si>
+    <t>PROTHIONAMIDE/ETHIONAMIDE (PTO/ETO)</t>
+  </si>
+  <si>
+    <t>a3820030-1c76-4251-8323-7f33f7f56761</t>
+  </si>
+  <si>
+    <t>74c78a90-ea77-43d6-a77e-ca4a55de65a7</t>
+  </si>
+  <si>
+    <t>c13bd24b-f54d-4d08-bcf5-9e1c4d60c3fb</t>
+  </si>
+  <si>
+    <t>ae1c0f6e-bf21-423c-a286-0e9cbf3e0a01</t>
   </si>
 </sst>
 </file>
@@ -2066,7 +2162,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91536433-8730-4EA0-BCCE-0E80DA08A6A5}">
-  <dimension ref="A1:Q227"/>
+  <dimension ref="A1:Q219"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
@@ -11659,10 +11755,10 @@
         <v>5</v>
       </c>
       <c r="C206" t="s">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="D206" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E206">
         <v>0</v>
@@ -11670,18 +11766,16 @@
       <c r="F206">
         <v>1</v>
       </c>
-      <c r="G206" t="s">
-        <v>36</v>
-      </c>
+      <c r="G206"/>
       <c r="H206">
         <v>109</v>
       </c>
       <c r="I206" t="str">
         <f>C206 &amp; " " &amp;L206</f>
-        <v xml:space="preserve">APPEARANCE OF SPECIMEN XPERT ULTRA</v>
+        <v xml:space="preserve">TUBERCULOSIS TEST RESULT DATE XPERT ULTRA</v>
       </c>
       <c r="J206" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="K206"/>
       <c r="L206" t="s">
@@ -11692,13 +11786,13 @@
         <v>1</v>
       </c>
       <c r="O206" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P206">
         <v>0</v>
       </c>
       <c r="Q206" t="s">
-        <v>414</v>
+        <v>442</v>
       </c>
     </row>
     <row r="207" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -11709,7 +11803,7 @@
         <v>5</v>
       </c>
       <c r="C207" t="s">
-        <v>51</v>
+        <v>443</v>
       </c>
       <c r="D207" t="s">
         <v>35</v>
@@ -11721,14 +11815,14 @@
         <v>1</v>
       </c>
       <c r="G207" t="s">
-        <v>52</v>
+        <v>418</v>
       </c>
       <c r="H207">
         <v>110</v>
       </c>
       <c r="I207" t="str">
         <f>C207 &amp; " " &amp;L207</f>
-        <v xml:space="preserve">MTB RESULT XPERT ULTRA</v>
+        <v xml:space="preserve">XPERT ULTRA RESULT XPERT ULTRA</v>
       </c>
       <c r="J207" t="s">
         <v>37</v>
@@ -11742,13 +11836,13 @@
         <v>1</v>
       </c>
       <c r="O207" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P207">
         <v>0</v>
       </c>
       <c r="Q207" t="s">
-        <v>415</v>
+        <v>444</v>
       </c>
     </row>
     <row r="208" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -11759,10 +11853,10 @@
         <v>5</v>
       </c>
       <c r="C208" t="s">
-        <v>85</v>
+        <v>445</v>
       </c>
       <c r="D208" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E208">
         <v>0</v>
@@ -11771,17 +11865,17 @@
         <v>1</v>
       </c>
       <c r="G208" t="s">
-        <v>45</v>
+        <v>446</v>
       </c>
       <c r="H208">
         <v>111</v>
       </c>
       <c r="I208" t="str">
         <f>C208 &amp; " " &amp;L208</f>
-        <v xml:space="preserve">ERROR CODE XPERT ULTRA</v>
+        <v xml:space="preserve">TEST NUMBER XPERT ULTRA</v>
       </c>
       <c r="J208" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="K208"/>
       <c r="L208" t="s">
@@ -11792,13 +11886,13 @@
         <v>1</v>
       </c>
       <c r="O208" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P208">
         <v>0</v>
       </c>
       <c r="Q208" t="s">
-        <v>416</v>
+        <v>447</v>
       </c>
     </row>
     <row r="209" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -11809,7 +11903,7 @@
         <v>5</v>
       </c>
       <c r="C209" t="s">
-        <v>417</v>
+        <v>448</v>
       </c>
       <c r="D209" t="s">
         <v>35</v>
@@ -11821,14 +11915,14 @@
         <v>1</v>
       </c>
       <c r="G209" t="s">
-        <v>418</v>
+        <v>449</v>
       </c>
       <c r="H209">
         <v>112</v>
       </c>
       <c r="I209" t="str">
         <f>C209 &amp; " " &amp;L209</f>
-        <v xml:space="preserve">XPERT ULTRA MTB BURDEN XPERT ULTRA</v>
+        <v xml:space="preserve">LAB XPERT ULTRA</v>
       </c>
       <c r="J209" t="s">
         <v>37</v>
@@ -11842,27 +11936,27 @@
         <v>1</v>
       </c>
       <c r="O209" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P209">
         <v>0</v>
       </c>
       <c r="Q209" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="210" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>209</v>
       </c>
-      <c r="B210" s="1">
+      <c r="B210">
         <v>5</v>
       </c>
       <c r="C210" t="s">
-        <v>171</v>
+        <v>81</v>
       </c>
       <c r="D210" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E210">
         <v>0</v>
@@ -11870,33 +11964,33 @@
       <c r="F210">
         <v>1</v>
       </c>
-      <c r="G210" t="s">
-        <v>62</v>
-      </c>
+      <c r="G210"/>
       <c r="H210">
         <v>113</v>
       </c>
       <c r="I210" t="str">
         <f>C210 &amp; " " &amp;L210</f>
-        <v xml:space="preserve">RIFAMPICIN RESULT XPERT ULTRA</v>
+        <v xml:space="preserve">TUBERCULOSIS TEST RESULT DATE XPERT XDR</v>
       </c>
       <c r="J210" t="s">
-        <v>37</v>
-      </c>
-      <c r="L210" s="1" t="s">
-        <v>413</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="K210"/>
+      <c r="L210" t="s">
+        <v>426</v>
+      </c>
+      <c r="M210"/>
       <c r="N210">
         <v>1</v>
       </c>
       <c r="O210" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P210">
         <v>0</v>
       </c>
       <c r="Q210" t="s">
-        <v>420</v>
+        <v>451</v>
       </c>
     </row>
     <row r="211" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -11907,10 +12001,10 @@
         <v>5</v>
       </c>
       <c r="C211" t="s">
-        <v>81</v>
+        <v>452</v>
       </c>
       <c r="D211" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E211">
         <v>0</v>
@@ -11918,33 +12012,35 @@
       <c r="F211">
         <v>1</v>
       </c>
-      <c r="G211"/>
+      <c r="G211" t="s">
+        <v>435</v>
+      </c>
       <c r="H211">
         <v>114</v>
       </c>
       <c r="I211" t="str">
         <f>C211 &amp; " " &amp;L211</f>
-        <v xml:space="preserve">TUBERCULOSIS TEST RESULT DATE XPERT ULTRA</v>
+        <v xml:space="preserve">XPERT XDR RESULT XPERT XDR</v>
       </c>
       <c r="J211" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="K211"/>
       <c r="L211" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="M211"/>
       <c r="N211">
         <v>1</v>
       </c>
       <c r="O211" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P211">
         <v>0</v>
       </c>
       <c r="Q211" t="s">
-        <v>421</v>
+        <v>453</v>
       </c>
     </row>
     <row r="212" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -11955,10 +12051,10 @@
         <v>5</v>
       </c>
       <c r="C212" t="s">
-        <v>279</v>
+        <v>454</v>
       </c>
       <c r="D212" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E212">
         <v>0</v>
@@ -11966,33 +12062,35 @@
       <c r="F212">
         <v>1</v>
       </c>
-      <c r="G212"/>
+      <c r="G212" t="s">
+        <v>455</v>
+      </c>
       <c r="H212">
         <v>115</v>
       </c>
       <c r="I212" t="str">
         <f>C212 &amp; " " &amp;L212</f>
-        <v xml:space="preserve">DATE OF SENDING TO CULTURE XPERT ULTRA</v>
+        <v xml:space="preserve">ISONIAZID (H) XPERT XDR</v>
       </c>
       <c r="J212" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="K212"/>
       <c r="L212" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="M212"/>
       <c r="N212">
         <v>1</v>
       </c>
       <c r="O212" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P212">
         <v>0</v>
       </c>
       <c r="Q212" t="s">
-        <v>422</v>
+        <v>456</v>
       </c>
     </row>
     <row r="213" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -12003,10 +12101,10 @@
         <v>5</v>
       </c>
       <c r="C213" t="s">
-        <v>280</v>
+        <v>457</v>
       </c>
       <c r="D213" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E213">
         <v>0</v>
@@ -12014,33 +12112,35 @@
       <c r="F213">
         <v>1</v>
       </c>
-      <c r="G213"/>
+      <c r="G213" t="s">
+        <v>458</v>
+      </c>
       <c r="H213">
         <v>116</v>
       </c>
       <c r="I213" t="str">
         <f>C213 &amp; " " &amp;L213</f>
-        <v xml:space="preserve">DATE OF SENDING TO DST XPERT ULTRA</v>
+        <v xml:space="preserve">FLUOROQUINOLONES (FQ) XPERT XDR</v>
       </c>
       <c r="J213" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="K213"/>
       <c r="L213" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="M213"/>
       <c r="N213">
         <v>1</v>
       </c>
       <c r="O213" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P213">
         <v>0</v>
       </c>
       <c r="Q213" t="s">
-        <v>423</v>
+        <v>459</v>
       </c>
     </row>
     <row r="214" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -12051,7 +12151,7 @@
         <v>5</v>
       </c>
       <c r="C214" t="s">
-        <v>282</v>
+        <v>460</v>
       </c>
       <c r="D214" t="s">
         <v>35</v>
@@ -12063,34 +12163,34 @@
         <v>1</v>
       </c>
       <c r="G214" t="s">
-        <v>295</v>
+        <v>461</v>
       </c>
       <c r="H214">
         <v>117</v>
       </c>
       <c r="I214" t="str">
         <f>C214 &amp; " " &amp;L214</f>
-        <v xml:space="preserve">SENT TO CULTURE XPERT ULTRA</v>
+        <v xml:space="preserve">AMIKACIN (AM) XPERT XDR</v>
       </c>
       <c r="J214" t="s">
         <v>37</v>
       </c>
       <c r="K214"/>
       <c r="L214" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="M214"/>
       <c r="N214">
         <v>1</v>
       </c>
       <c r="O214" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P214">
         <v>0</v>
       </c>
       <c r="Q214" t="s">
-        <v>424</v>
+        <v>462</v>
       </c>
     </row>
     <row r="215" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -12101,7 +12201,7 @@
         <v>5</v>
       </c>
       <c r="C215" t="s">
-        <v>281</v>
+        <v>463</v>
       </c>
       <c r="D215" t="s">
         <v>35</v>
@@ -12113,34 +12213,34 @@
         <v>1</v>
       </c>
       <c r="G215" t="s">
-        <v>294</v>
+        <v>464</v>
       </c>
       <c r="H215">
         <v>118</v>
       </c>
       <c r="I215" t="str">
         <f>C215 &amp; " " &amp;L215</f>
-        <v xml:space="preserve">SENT TO DST XPERT ULTRA</v>
+        <v xml:space="preserve">CAPREOMYCIN (CM) XPERT XDR</v>
       </c>
       <c r="J215" t="s">
         <v>37</v>
       </c>
       <c r="K215"/>
       <c r="L215" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="M215"/>
       <c r="N215">
         <v>1</v>
       </c>
       <c r="O215" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P215">
         <v>0</v>
       </c>
       <c r="Q215" t="s">
-        <v>425</v>
+        <v>465</v>
       </c>
     </row>
     <row r="216" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -12151,7 +12251,7 @@
         <v>5</v>
       </c>
       <c r="C216" t="s">
-        <v>34</v>
+        <v>466</v>
       </c>
       <c r="D216" t="s">
         <v>35</v>
@@ -12163,14 +12263,14 @@
         <v>1</v>
       </c>
       <c r="G216" t="s">
-        <v>36</v>
+        <v>467</v>
       </c>
       <c r="H216">
         <v>119</v>
       </c>
       <c r="I216" t="str">
         <f>C216 &amp; " " &amp;L216</f>
-        <v xml:space="preserve">APPEARANCE OF SPECIMEN XPERT XDR</v>
+        <v xml:space="preserve">KANAMYCIN (KM) XPERT XDR</v>
       </c>
       <c r="J216" t="s">
         <v>37</v>
@@ -12184,13 +12284,13 @@
         <v>1</v>
       </c>
       <c r="O216" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P216">
         <v>0</v>
       </c>
       <c r="Q216" t="s">
-        <v>427</v>
+        <v>468</v>
       </c>
     </row>
     <row r="217" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -12201,7 +12301,7 @@
         <v>5</v>
       </c>
       <c r="C217" t="s">
-        <v>51</v>
+        <v>469</v>
       </c>
       <c r="D217" t="s">
         <v>35</v>
@@ -12213,14 +12313,14 @@
         <v>1</v>
       </c>
       <c r="G217" t="s">
-        <v>52</v>
+        <v>470</v>
       </c>
       <c r="H217">
         <v>120</v>
       </c>
       <c r="I217" t="str">
         <f>C217 &amp; " " &amp;L217</f>
-        <v xml:space="preserve">MTB RESULT XPERT XDR</v>
+        <v xml:space="preserve">PROTHIONAMIDE/ETHIONAMIDE (PTO/ETO) XPERT XDR</v>
       </c>
       <c r="J217" t="s">
         <v>37</v>
@@ -12234,13 +12334,13 @@
         <v>1</v>
       </c>
       <c r="O217" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P217">
         <v>0</v>
       </c>
       <c r="Q217" t="s">
-        <v>428</v>
+        <v>471</v>
       </c>
     </row>
     <row r="218" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -12251,10 +12351,10 @@
         <v>5</v>
       </c>
       <c r="C218" t="s">
-        <v>85</v>
+        <v>445</v>
       </c>
       <c r="D218" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E218">
         <v>0</v>
@@ -12263,17 +12363,17 @@
         <v>1</v>
       </c>
       <c r="G218" t="s">
-        <v>45</v>
+        <v>446</v>
       </c>
       <c r="H218">
         <v>121</v>
       </c>
       <c r="I218" t="str">
         <f>C218 &amp; " " &amp;L218</f>
-        <v xml:space="preserve">ERROR CODE XPERT XDR</v>
+        <v xml:space="preserve">TEST NUMBER XPERT XDR</v>
       </c>
       <c r="J218" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="K218"/>
       <c r="L218" t="s">
@@ -12284,24 +12384,24 @@
         <v>1</v>
       </c>
       <c r="O218" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P218">
         <v>0</v>
       </c>
       <c r="Q218" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="219" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>218</v>
       </c>
-      <c r="B219" s="1">
+      <c r="B219">
         <v>5</v>
       </c>
       <c r="C219" t="s">
-        <v>170</v>
+        <v>448</v>
       </c>
       <c r="D219" t="s">
         <v>35</v>
@@ -12313,425 +12413,39 @@
         <v>1</v>
       </c>
       <c r="G219" t="s">
-        <v>88</v>
+        <v>449</v>
       </c>
       <c r="H219">
         <v>122</v>
       </c>
       <c r="I219" t="str">
         <f>C219 &amp; " " &amp;L219</f>
-        <v xml:space="preserve">ISONIAZID RESULT XPERT XDR</v>
+        <v xml:space="preserve">LAB XPERT XDR</v>
       </c>
       <c r="J219" t="s">
         <v>37</v>
       </c>
-      <c r="L219" s="1" t="s">
+      <c r="K219"/>
+      <c r="L219" t="s">
         <v>426</v>
       </c>
+      <c r="M219"/>
       <c r="N219">
         <v>1</v>
       </c>
       <c r="O219" s="4">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="P219">
         <v>0</v>
       </c>
       <c r="Q219" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A220">
-        <v>219</v>
-      </c>
-      <c r="B220">
-        <v>5</v>
-      </c>
-      <c r="C220" s="8" t="s">
-        <v>307</v>
-      </c>
-      <c r="D220" t="s">
-        <v>35</v>
-      </c>
-      <c r="E220">
-        <v>0</v>
-      </c>
-      <c r="F220">
-        <v>1</v>
-      </c>
-      <c r="G220" t="s">
-        <v>289</v>
-      </c>
-      <c r="H220">
-        <v>123</v>
-      </c>
-      <c r="I220" t="str">
-        <f>C220 &amp; " " &amp;L220</f>
-        <v xml:space="preserve">MOX/OFX RESULT XPERT XDR</v>
-      </c>
-      <c r="J220" t="s">
-        <v>37</v>
-      </c>
-      <c r="L220" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="N220">
-        <v>1</v>
-      </c>
-      <c r="O220" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P220">
-        <v>0</v>
-      </c>
-      <c r="Q220" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="221" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A221">
-        <v>220</v>
-      </c>
-      <c r="B221">
-        <v>5</v>
-      </c>
-      <c r="C221" s="8" t="s">
-        <v>432</v>
-      </c>
-      <c r="D221" t="s">
-        <v>35</v>
-      </c>
-      <c r="E221">
-        <v>0</v>
-      </c>
-      <c r="F221">
-        <v>1</v>
-      </c>
-      <c r="G221" t="s">
-        <v>288</v>
-      </c>
-      <c r="H221">
-        <v>124</v>
-      </c>
-      <c r="I221" t="str">
-        <f>C221 &amp; " " &amp;L221</f>
-        <v xml:space="preserve">KM/AM/CM RESULT XPERT XDR</v>
-      </c>
-      <c r="J221" t="s">
-        <v>37</v>
-      </c>
-      <c r="L221" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="N221">
-        <v>1</v>
-      </c>
-      <c r="O221" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P221">
-        <v>0</v>
-      </c>
-      <c r="Q221" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="222" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A222">
-        <v>221</v>
-      </c>
-      <c r="B222" s="1">
-        <v>5</v>
-      </c>
-      <c r="C222" t="s">
-        <v>434</v>
-      </c>
-      <c r="D222" t="s">
-        <v>35</v>
-      </c>
-      <c r="E222">
-        <v>0</v>
-      </c>
-      <c r="F222">
-        <v>1</v>
-      </c>
-      <c r="G222" t="s">
-        <v>435</v>
-      </c>
-      <c r="H222">
-        <v>125</v>
-      </c>
-      <c r="I222" t="str">
-        <f>C222 &amp; " " &amp;L222</f>
-        <v xml:space="preserve">ETHIONAMIDE RESULT XPERT XDR</v>
-      </c>
-      <c r="J222" t="s">
-        <v>37</v>
-      </c>
-      <c r="L222" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="N222">
-        <v>1</v>
-      </c>
-      <c r="O222" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P222">
-        <v>0</v>
-      </c>
-      <c r="Q222" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="223" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A223">
-        <v>222</v>
-      </c>
-      <c r="B223">
-        <v>5</v>
-      </c>
-      <c r="C223" t="s">
-        <v>81</v>
-      </c>
-      <c r="D223" t="s">
-        <v>39</v>
-      </c>
-      <c r="E223">
-        <v>0</v>
-      </c>
-      <c r="F223">
-        <v>1</v>
-      </c>
-      <c r="G223"/>
-      <c r="H223">
-        <v>126</v>
-      </c>
-      <c r="I223" t="str">
-        <f>C223 &amp; " " &amp;L223</f>
-        <v xml:space="preserve">TUBERCULOSIS TEST RESULT DATE XPERT XDR</v>
-      </c>
-      <c r="J223" t="s">
-        <v>41</v>
-      </c>
-      <c r="K223"/>
-      <c r="L223" t="s">
-        <v>426</v>
-      </c>
-      <c r="M223"/>
-      <c r="N223">
-        <v>1</v>
-      </c>
-      <c r="O223" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P223">
-        <v>0</v>
-      </c>
-      <c r="Q223" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="224" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A224">
-        <v>223</v>
-      </c>
-      <c r="B224">
-        <v>5</v>
-      </c>
-      <c r="C224" t="s">
-        <v>279</v>
-      </c>
-      <c r="D224" t="s">
-        <v>39</v>
-      </c>
-      <c r="E224">
-        <v>0</v>
-      </c>
-      <c r="F224">
-        <v>1</v>
-      </c>
-      <c r="G224"/>
-      <c r="H224">
-        <v>127</v>
-      </c>
-      <c r="I224" t="str">
-        <f>C224 &amp; " " &amp;L224</f>
-        <v xml:space="preserve">DATE OF SENDING TO CULTURE XPERT XDR</v>
-      </c>
-      <c r="J224" t="s">
-        <v>41</v>
-      </c>
-      <c r="K224"/>
-      <c r="L224" t="s">
-        <v>426</v>
-      </c>
-      <c r="M224"/>
-      <c r="N224">
-        <v>1</v>
-      </c>
-      <c r="O224" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P224">
-        <v>0</v>
-      </c>
-      <c r="Q224" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="225" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A225">
-        <v>224</v>
-      </c>
-      <c r="B225">
-        <v>5</v>
-      </c>
-      <c r="C225" t="s">
-        <v>280</v>
-      </c>
-      <c r="D225" t="s">
-        <v>39</v>
-      </c>
-      <c r="E225">
-        <v>0</v>
-      </c>
-      <c r="F225">
-        <v>1</v>
-      </c>
-      <c r="G225"/>
-      <c r="H225">
-        <v>128</v>
-      </c>
-      <c r="I225" t="str">
-        <f>C225 &amp; " " &amp;L225</f>
-        <v xml:space="preserve">DATE OF SENDING TO DST XPERT XDR</v>
-      </c>
-      <c r="J225" t="s">
-        <v>41</v>
-      </c>
-      <c r="K225"/>
-      <c r="L225" t="s">
-        <v>426</v>
-      </c>
-      <c r="M225"/>
-      <c r="N225">
-        <v>1</v>
-      </c>
-      <c r="O225" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P225">
-        <v>0</v>
-      </c>
-      <c r="Q225" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="226" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A226">
-        <v>225</v>
-      </c>
-      <c r="B226">
-        <v>5</v>
-      </c>
-      <c r="C226" t="s">
-        <v>282</v>
-      </c>
-      <c r="D226" t="s">
-        <v>35</v>
-      </c>
-      <c r="E226">
-        <v>0</v>
-      </c>
-      <c r="F226">
-        <v>1</v>
-      </c>
-      <c r="G226" t="s">
-        <v>295</v>
-      </c>
-      <c r="H226">
-        <v>129</v>
-      </c>
-      <c r="I226" t="str">
-        <f>C226 &amp; " " &amp;L226</f>
-        <v xml:space="preserve">SENT TO CULTURE XPERT XDR</v>
-      </c>
-      <c r="J226" t="s">
-        <v>37</v>
-      </c>
-      <c r="K226"/>
-      <c r="L226" t="s">
-        <v>426</v>
-      </c>
-      <c r="M226"/>
-      <c r="N226">
-        <v>1</v>
-      </c>
-      <c r="O226" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P226">
-        <v>0</v>
-      </c>
-      <c r="Q226" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="227" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A227">
-        <v>226</v>
-      </c>
-      <c r="B227">
-        <v>5</v>
-      </c>
-      <c r="C227" t="s">
-        <v>281</v>
-      </c>
-      <c r="D227" t="s">
-        <v>35</v>
-      </c>
-      <c r="E227">
-        <v>0</v>
-      </c>
-      <c r="F227">
-        <v>1</v>
-      </c>
-      <c r="G227" t="s">
-        <v>294</v>
-      </c>
-      <c r="H227">
-        <v>130</v>
-      </c>
-      <c r="I227" t="str">
-        <f>C227 &amp; " " &amp;L227</f>
-        <v xml:space="preserve">SENT TO DST XPERT XDR</v>
-      </c>
-      <c r="J227" t="s">
-        <v>37</v>
-      </c>
-      <c r="K227"/>
-      <c r="L227" t="s">
-        <v>426</v>
-      </c>
-      <c r="M227"/>
-      <c r="N227">
-        <v>1</v>
-      </c>
-      <c r="O227" s="4">
-        <v>46313</v>
-      </c>
-      <c r="P227">
-        <v>0</v>
-      </c>
-      <c r="Q227" t="s">
-        <v>441</v>
+        <v>473</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q227" xr:uid="{91536433-8730-4EA0-BCCE-0E80DA08A6A5}"/>
-  <conditionalFormatting sqref="Q2:Q227">
+  <autoFilter ref="A1:Q219" xr:uid="{91536433-8730-4EA0-BCCE-0E80DA08A6A5}"/>
+  <conditionalFormatting sqref="Q2:Q219">
     <cfRule type="duplicateValues" dxfId="0" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>